<commit_message>
Juli 2026: rekordmaaned, 1461 signups
</commit_message>
<xml_diff>
--- a/AE-marketingrapport-master.xlsx
+++ b/AE-marketingrapport-master.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="233">
   <si>
     <t xml:space="preserve">KONFIGURATION</t>
   </si>
@@ -388,6 +388,9 @@
     <t xml:space="preserve">Konverteringen stiger for anden måned i træk, og churn normaliseres efter maj-toppen.</t>
   </si>
   <si>
+    <t xml:space="preserve">Juli sætter rekord: 1.461 signups og 10 pct. konvertering midt i lavsæsonen.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hvad skete der (2-3 sætn.)</t>
   </si>
   <si>
@@ -397,6 +400,9 @@
     <t xml:space="preserve">Sign-ups landede på 984, et forventet sæsonfald fra maj (1.035), men konverteringen steg igen — blended CVR ramte 6,4% mod 5,8% i maj. Google leverede 74 kunder til en CAC på 133 kr. (kanalens næstbedste måned), og Brand search fastholdt det høje niveau med 446 kunder. Churn faldt tilbage fra 2,6% til 2,2%, og vi rundede 13.318 aktive kunder (+582).</t>
   </si>
   <si>
+    <t xml:space="preserve">Juli blev den største måned i Altid Energis historie med 1.461 signups, klart over den tidligere rekord på 1.300 fra februar. Blended konvertering ramte 10,0 pct. (ny rekord), og blended CAC faldt til 131 kr. fra 157 kr. Brand search leverede 733 kunder (rekord), Google sin bedste konverteringsmåned (CVR 11,1 pct., CAC 105 kr.), og affiliates voksede til 334 kunder. Aktive kunder rundede 13.970 (+652), og churn holdt sig stabil på 2,2 pct.</t>
+  </si>
+  <si>
     <t xml:space="preserve">WINS — HVAD VIRKEDE</t>
   </si>
   <si>
@@ -409,6 +415,9 @@
     <t xml:space="preserve">Blended CVR ramte 6,4% — anden stigning i træk (3,8% → 5,8% → 6,4%) på trods af lavere trafik.</t>
   </si>
   <si>
+    <t xml:space="preserve">1.461 signups, den højeste måned nogensinde (tidligere rekord 1.300 i februar), leveret midt i sommerlavsæsonen.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Win 2</t>
   </si>
   <si>
@@ -418,6 +427,9 @@
     <t xml:space="preserve">Churn faldt fra maj's rekordhøje 2,6% til 2,2%, og aktive kunder rundede 13.318 (+582 netto).</t>
   </si>
   <si>
+    <t xml:space="preserve">Blended CVR ramte 10,0 pct. (rekord), og blended CAC faldt til 131 kr. fra 157 kr.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Win 3</t>
   </si>
   <si>
@@ -427,6 +439,9 @@
     <t xml:space="preserve">Google leverede 74 kunder (næstbedste måned nogensinde) til CAC 133 kr., og Brand search fastholdt momentum med 446 kunder.</t>
   </si>
   <si>
+    <t xml:space="preserve">Brand search satte rekord med 733 kunder, og Meta CAC faldt til 252 kr. fra 561 kr. efter optimeringen mod køb.</t>
+  </si>
+  <si>
     <t xml:space="preserve">WATCH-OUTS — OBS OMRÅDER</t>
   </si>
   <si>
@@ -439,6 +454,9 @@
     <t xml:space="preserve">Meta-CAC steg til 561 kr. (fra 432 kr.) — et normalt sæsonmønster, når efterspørgslen falder hen over sommeren. 80 kunder i lavsæsonen er reelt bedre end forventet.</t>
   </si>
   <si>
+    <t xml:space="preserve">Organisk trafik lå på 3.640 klik, fortsat sommerlavt. 389.000 eksponeringer viser dog stærk synlighed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Watch 2</t>
   </si>
   <si>
@@ -466,6 +484,9 @@
     <t xml:space="preserve">Konverteringsarbejdet på hjemmesiden virker: blended CVR er steget to måneder i træk (3,8% → 5,8% → 6,4%) på trods af lavere trafik. Volumen — ikke konvertering — er nu den primære begrænsning ind i sommerens lavsæson.</t>
   </si>
   <si>
+    <t xml:space="preserve">Efterspørgslen fra de 32.500 tvangsflyttede elkunder ramte direkte ned i et optimeret setup: rekordhøj brand search, stigende konvertering og faldende CAC på samme tid. Volumen kom tilbage langt tidligere end ventet i lavsæsonen.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Markedsnote / konkurrence</t>
   </si>
   <si>
@@ -473,6 +494,9 @@
   </si>
   <si>
     <t xml:space="preserve">32.500 danske elkunder tvangsflyttes fra deres nuværende leverandører.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32.500 danske elkunder er tvangsflyttet fra deres leverandører i sommerens løb.</t>
   </si>
   <si>
     <t xml:space="preserve">NEXT MONTH FOCUS</t>
@@ -2105,8 +2129,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="94899266"/>
-        <c:axId val="49404710"/>
+        <c:axId val="86917899"/>
+        <c:axId val="31025123"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2291,11 +2315,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="98418137"/>
-        <c:axId val="9044728"/>
+        <c:axId val="4644969"/>
+        <c:axId val="16117395"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="94899266"/>
+        <c:axId val="86917899"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2326,7 +2350,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49404710"/>
+        <c:crossAx val="31025123"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -2334,7 +2358,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="49404710"/>
+        <c:axId val="31025123"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2399,12 +2423,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94899266"/>
+        <c:crossAx val="86917899"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:dateAx>
-        <c:axId val="98418137"/>
+        <c:axId val="4644969"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2435,7 +2459,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9044728"/>
+        <c:crossAx val="16117395"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -2443,7 +2467,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="9044728"/>
+        <c:axId val="16117395"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2508,7 +2532,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98418137"/>
+        <c:crossAx val="4644969"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2723,11 +2747,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52091142"/>
-        <c:axId val="42690782"/>
+        <c:axId val="71657506"/>
+        <c:axId val="24797220"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52091142"/>
+        <c:axId val="71657506"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2758,7 +2782,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42690782"/>
+        <c:crossAx val="24797220"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2766,7 +2790,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42690782"/>
+        <c:axId val="24797220"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2797,7 +2821,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52091142"/>
+        <c:crossAx val="71657506"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2988,11 +3012,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="37218380"/>
-        <c:axId val="63489669"/>
+        <c:axId val="84131102"/>
+        <c:axId val="57461450"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="37218380"/>
+        <c:axId val="84131102"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3023,7 +3047,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63489669"/>
+        <c:crossAx val="57461450"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3031,7 +3055,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63489669"/>
+        <c:axId val="57461450"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3071,7 +3095,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37218380"/>
+        <c:crossAx val="84131102"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3323,11 +3347,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="17437926"/>
-        <c:axId val="61543854"/>
+        <c:axId val="78426142"/>
+        <c:axId val="93029554"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="17437926"/>
+        <c:axId val="78426142"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3358,7 +3382,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61543854"/>
+        <c:crossAx val="93029554"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -3366,7 +3390,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="61543854"/>
+        <c:axId val="93029554"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3397,7 +3421,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17437926"/>
+        <c:crossAx val="78426142"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3649,11 +3673,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="59890267"/>
-        <c:axId val="66000661"/>
+        <c:axId val="46415980"/>
+        <c:axId val="59975435"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="59890267"/>
+        <c:axId val="46415980"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3684,7 +3708,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66000661"/>
+        <c:crossAx val="59975435"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -3692,7 +3716,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="66000661"/>
+        <c:axId val="59975435"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3723,7 +3747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59890267"/>
+        <c:crossAx val="46415980"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3762,9 +3786,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
-      <xdr:colOff>224280</xdr:colOff>
+      <xdr:colOff>221760</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>104400</xdr:rowOff>
+      <xdr:rowOff>101880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3773,7 +3797,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="293400" y="2114640"/>
-        <a:ext cx="9636120" cy="2333160"/>
+        <a:ext cx="9633600" cy="2330640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3792,9 +3816,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>234360</xdr:colOff>
+      <xdr:colOff>231840</xdr:colOff>
       <xdr:row>81</xdr:row>
-      <xdr:rowOff>66240</xdr:rowOff>
+      <xdr:rowOff>63720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3803,7 +3827,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="293400" y="11458440"/>
-        <a:ext cx="4635000" cy="2333160"/>
+        <a:ext cx="4632480" cy="2330640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3822,9 +3846,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>234720</xdr:colOff>
+      <xdr:colOff>232200</xdr:colOff>
       <xdr:row>81</xdr:row>
-      <xdr:rowOff>66240</xdr:rowOff>
+      <xdr:rowOff>63720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3833,7 +3857,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4694040" y="11458440"/>
-        <a:ext cx="4635000" cy="2333160"/>
+        <a:ext cx="4632480" cy="2330640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3852,9 +3876,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>234360</xdr:colOff>
+      <xdr:colOff>231840</xdr:colOff>
       <xdr:row>123</xdr:row>
-      <xdr:rowOff>153720</xdr:rowOff>
+      <xdr:rowOff>151200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3863,7 +3887,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="293400" y="18773640"/>
-        <a:ext cx="4635000" cy="1611360"/>
+        <a:ext cx="4632480" cy="1608840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3882,9 +3906,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>234720</xdr:colOff>
+      <xdr:colOff>232200</xdr:colOff>
       <xdr:row>123</xdr:row>
-      <xdr:rowOff>153720</xdr:rowOff>
+      <xdr:rowOff>151200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3893,7 +3917,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4694040" y="18773640"/>
-        <a:ext cx="4635000" cy="1611360"/>
+        <a:ext cx="4632480" cy="1608840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4602,7 +4626,9 @@
       <c r="Y5" s="26" t="n">
         <v>44861</v>
       </c>
-      <c r="Z5" s="26"/>
+      <c r="Z5" s="26" t="n">
+        <v>15618</v>
+      </c>
       <c r="AA5" s="26"/>
       <c r="AB5" s="26"/>
       <c r="AC5" s="26"/>
@@ -4682,7 +4708,9 @@
       <c r="Y6" s="26" t="n">
         <v>545000</v>
       </c>
-      <c r="Z6" s="26"/>
+      <c r="Z6" s="26" t="n">
+        <v>191437</v>
+      </c>
       <c r="AA6" s="26"/>
       <c r="AB6" s="26"/>
       <c r="AC6" s="26"/>
@@ -4762,7 +4790,9 @@
       <c r="Y7" s="26" t="n">
         <v>3658</v>
       </c>
-      <c r="Z7" s="26"/>
+      <c r="Z7" s="26" t="n">
+        <v>1392</v>
+      </c>
       <c r="AA7" s="26"/>
       <c r="AB7" s="26"/>
       <c r="AC7" s="26"/>
@@ -4842,7 +4872,9 @@
       <c r="Y8" s="26" t="n">
         <v>80</v>
       </c>
-      <c r="Z8" s="26"/>
+      <c r="Z8" s="26" t="n">
+        <v>62</v>
+      </c>
       <c r="AA8" s="26"/>
       <c r="AB8" s="26"/>
       <c r="AC8" s="26"/>
@@ -4946,7 +4978,7 @@
       </c>
       <c r="Z9" s="27" t="n">
         <f aca="false">IFERROR(Z8/Z7,0)</f>
-        <v>0</v>
+        <v>0.0445402298850575</v>
       </c>
       <c r="AA9" s="27" t="n">
         <f aca="false">IFERROR(AA8/AA7,0)</f>
@@ -5075,7 +5107,7 @@
       </c>
       <c r="Z10" s="28" t="n">
         <f aca="false">IFERROR(Z5/Z8,0)</f>
-        <v>0</v>
+        <v>251.903225806452</v>
       </c>
       <c r="AA10" s="28" t="n">
         <f aca="false">IFERROR(AA5/AA8,0)</f>
@@ -5163,7 +5195,9 @@
       <c r="Y12" s="26" t="n">
         <v>9860</v>
       </c>
-      <c r="Z12" s="26"/>
+      <c r="Z12" s="26" t="n">
+        <v>6079</v>
+      </c>
       <c r="AA12" s="26"/>
       <c r="AB12" s="26"/>
       <c r="AC12" s="26"/>
@@ -5223,7 +5257,9 @@
       <c r="Y13" s="26" t="n">
         <v>18000</v>
       </c>
-      <c r="Z13" s="26"/>
+      <c r="Z13" s="26" t="n">
+        <v>10756</v>
+      </c>
       <c r="AA13" s="26"/>
       <c r="AB13" s="26"/>
       <c r="AC13" s="26"/>
@@ -5283,7 +5319,9 @@
       <c r="Y14" s="26" t="n">
         <v>910</v>
       </c>
-      <c r="Z14" s="26"/>
+      <c r="Z14" s="26" t="n">
+        <v>522</v>
+      </c>
       <c r="AA14" s="26"/>
       <c r="AB14" s="26"/>
       <c r="AC14" s="26"/>
@@ -5343,7 +5381,9 @@
       <c r="Y15" s="26" t="n">
         <v>74</v>
       </c>
-      <c r="Z15" s="26"/>
+      <c r="Z15" s="26" t="n">
+        <v>58</v>
+      </c>
       <c r="AA15" s="26"/>
       <c r="AB15" s="26"/>
       <c r="AC15" s="26"/>
@@ -5447,7 +5487,7 @@
       </c>
       <c r="Z16" s="27" t="n">
         <f aca="false">IFERROR(Z15/Z14,0)</f>
-        <v>0</v>
+        <v>0.111111111111111</v>
       </c>
       <c r="AA16" s="27" t="n">
         <f aca="false">IFERROR(AA15/AA14,0)</f>
@@ -5576,7 +5616,7 @@
       </c>
       <c r="Z17" s="28" t="n">
         <f aca="false">IFERROR(Z12/Z15,0)</f>
-        <v>0</v>
+        <v>104.810344827586</v>
       </c>
       <c r="AA17" s="28" t="n">
         <f aca="false">IFERROR(AA12/AA15,0)</f>
@@ -6534,7 +6574,9 @@
       <c r="Y33" s="26" t="n">
         <v>1322</v>
       </c>
-      <c r="Z33" s="26"/>
+      <c r="Z33" s="26" t="n">
+        <v>2037</v>
+      </c>
       <c r="AA33" s="26"/>
       <c r="AB33" s="26"/>
       <c r="AC33" s="26"/>
@@ -6610,7 +6652,9 @@
       <c r="Y34" s="26" t="n">
         <v>8311</v>
       </c>
-      <c r="Z34" s="26"/>
+      <c r="Z34" s="26" t="n">
+        <v>9641</v>
+      </c>
       <c r="AA34" s="26"/>
       <c r="AB34" s="26"/>
       <c r="AC34" s="26"/>
@@ -6690,7 +6734,9 @@
       <c r="Y35" s="26" t="n">
         <v>3761</v>
       </c>
-      <c r="Z35" s="26"/>
+      <c r="Z35" s="26" t="n">
+        <v>4746</v>
+      </c>
       <c r="AA35" s="26"/>
       <c r="AB35" s="26"/>
       <c r="AC35" s="26"/>
@@ -6770,7 +6816,9 @@
       <c r="Y36" s="26" t="n">
         <v>446</v>
       </c>
-      <c r="Z36" s="26"/>
+      <c r="Z36" s="26" t="n">
+        <v>733</v>
+      </c>
       <c r="AA36" s="26"/>
       <c r="AB36" s="26"/>
       <c r="AC36" s="26"/>
@@ -6874,7 +6922,7 @@
       </c>
       <c r="Z37" s="27" t="n">
         <f aca="false">IFERROR(Z36/Z35,0)</f>
-        <v>0</v>
+        <v>0.154445849136115</v>
       </c>
       <c r="AA37" s="27" t="n">
         <f aca="false">IFERROR(AA36/AA35,0)</f>
@@ -7003,7 +7051,7 @@
       </c>
       <c r="Z38" s="28" t="n">
         <f aca="false">IFERROR(Z33/Z36,0)</f>
-        <v>0</v>
+        <v>2.77899045020464</v>
       </c>
       <c r="AA38" s="28" t="n">
         <f aca="false">IFERROR(AA33/AA36,0)</f>
@@ -7543,7 +7591,9 @@
       <c r="Y48" s="26" t="n">
         <v>98500</v>
       </c>
-      <c r="Z48" s="26"/>
+      <c r="Z48" s="26" t="n">
+        <v>167000</v>
+      </c>
       <c r="AA48" s="26"/>
       <c r="AB48" s="26"/>
       <c r="AC48" s="26"/>
@@ -7647,7 +7697,9 @@
       <c r="Y50" s="26" t="n">
         <v>2225</v>
       </c>
-      <c r="Z50" s="26"/>
+      <c r="Z50" s="26" t="n">
+        <v>4278</v>
+      </c>
       <c r="AA50" s="26"/>
       <c r="AB50" s="26"/>
       <c r="AC50" s="26"/>
@@ -7709,7 +7761,9 @@
       <c r="Y51" s="26" t="n">
         <v>197</v>
       </c>
-      <c r="Z51" s="26"/>
+      <c r="Z51" s="26" t="n">
+        <v>334</v>
+      </c>
       <c r="AA51" s="26"/>
       <c r="AB51" s="26"/>
       <c r="AC51" s="26"/>
@@ -7813,7 +7867,7 @@
       </c>
       <c r="Z52" s="27" t="n">
         <f aca="false">IFERROR(Z51/Z50,0)</f>
-        <v>0</v>
+        <v>0.0780738662926601</v>
       </c>
       <c r="AA52" s="27" t="n">
         <f aca="false">IFERROR(AA51/AA50,0)</f>
@@ -7942,7 +7996,7 @@
       </c>
       <c r="Z53" s="28" t="n">
         <f aca="false">IFERROR(Z48/Z51,0)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="AA53" s="28" t="n">
         <f aca="false">IFERROR(AA48/AA51,0)</f>
@@ -9765,7 +9819,9 @@
       <c r="Y86" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Z86" s="26"/>
+      <c r="Z86" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="AA86" s="26"/>
       <c r="AB86" s="26"/>
       <c r="AC86" s="26"/>
@@ -9805,7 +9861,9 @@
       <c r="Y87" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Z87" s="26"/>
+      <c r="Z87" s="26" t="n">
+        <v>389000</v>
+      </c>
       <c r="AA87" s="26"/>
       <c r="AB87" s="26"/>
       <c r="AC87" s="26"/>
@@ -9871,7 +9929,9 @@
       <c r="Y88" s="26" t="n">
         <v>4800</v>
       </c>
-      <c r="Z88" s="26"/>
+      <c r="Z88" s="26" t="n">
+        <v>3640</v>
+      </c>
       <c r="AA88" s="26"/>
       <c r="AB88" s="26"/>
       <c r="AC88" s="26"/>
@@ -9921,7 +9981,9 @@
       <c r="Y89" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="Z89" s="26"/>
+      <c r="Z89" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="AA89" s="26"/>
       <c r="AB89" s="26"/>
       <c r="AC89" s="26"/>
@@ -11463,7 +11525,7 @@
       </c>
       <c r="Z110" s="33" t="n">
         <f aca="false">Z5+Z12+Z19+Z26+Z33+Z41+Z48+Z56+Z63+Z71+Z78+Z86</f>
-        <v>0</v>
+        <v>190734</v>
       </c>
       <c r="AA110" s="33" t="n">
         <f aca="false">AA5+AA12+AA19+AA26+AA33+AA41+AA48+AA56+AA63+AA71+AA78+AA86</f>
@@ -11592,7 +11654,7 @@
       </c>
       <c r="Z111" s="33" t="n">
         <f aca="false">Z8+Z15+Z22+Z29+Z36+Z44+Z51+Z59+Z66+Z74+Z81+Z89</f>
-        <v>0</v>
+        <v>1187</v>
       </c>
       <c r="AA111" s="33" t="n">
         <f aca="false">AA8+AA15+AA22+AA29+AA36+AA44+AA51+AA59+AA66+AA74+AA81+AA89</f>
@@ -11721,7 +11783,7 @@
       </c>
       <c r="Z112" s="33" t="n">
         <f aca="false">IFERROR(Z110/Z111,0)</f>
-        <v>0</v>
+        <v>160.685762426285</v>
       </c>
       <c r="AA112" s="33" t="n">
         <f aca="false">IFERROR(AA110/AA111,0)</f>
@@ -11850,7 +11912,7 @@
       </c>
       <c r="Z113" s="33" t="n">
         <f aca="false">Z7+Z14+Z21+Z28+Z35+Z43+Z50+Z58+Z65+Z73+Z80+Z88</f>
-        <v>0</v>
+        <v>14578</v>
       </c>
       <c r="AA113" s="33" t="n">
         <f aca="false">AA7+AA14+AA21+AA28+AA35+AA43+AA50+AA58+AA65+AA73+AA80+AA88</f>
@@ -11979,7 +12041,7 @@
       </c>
       <c r="Z114" s="33" t="n">
         <f aca="false">Z7+Z14+Z21+Z28+Z35+Z43+Z50+Z58+Z65+Z73+Z80</f>
-        <v>0</v>
+        <v>10938</v>
       </c>
       <c r="AA114" s="33" t="n">
         <f aca="false">AA7+AA14+AA21+AA28+AA35+AA43+AA50+AA58+AA65+AA73+AA80</f>
@@ -12108,7 +12170,7 @@
       </c>
       <c r="Z115" s="33" t="n">
         <f aca="false">Z88</f>
-        <v>0</v>
+        <v>3640</v>
       </c>
       <c r="AA115" s="33" t="n">
         <f aca="false">AA88</f>
@@ -12237,7 +12299,7 @@
       </c>
       <c r="Z116" s="34" t="n">
         <f aca="false">IFERROR(Z111/Z113,0)</f>
-        <v>0</v>
+        <v>0.0814240636575662</v>
       </c>
       <c r="AA116" s="34" t="n">
         <f aca="false">IFERROR(AA111/AA113,0)</f>
@@ -12366,7 +12428,7 @@
       </c>
       <c r="Z117" s="33" t="n">
         <f aca="false">Z5+Z12+Z19+Z26+Z33</f>
-        <v>0</v>
+        <v>23734</v>
       </c>
       <c r="AA117" s="33" t="n">
         <f aca="false">AA5+AA12+AA19+AA26+AA33</f>
@@ -12495,7 +12557,7 @@
       </c>
       <c r="Z118" s="33" t="n">
         <f aca="false">Z8+Z15+Z22+Z29+Z36</f>
-        <v>0</v>
+        <v>853</v>
       </c>
       <c r="AA118" s="33" t="n">
         <f aca="false">AA8+AA15+AA22+AA29+AA36</f>
@@ -12624,7 +12686,7 @@
       </c>
       <c r="Z119" s="33" t="n">
         <f aca="false">IFERROR(Z117/Z118,0)</f>
-        <v>0</v>
+        <v>27.8241500586167</v>
       </c>
       <c r="AA119" s="33" t="n">
         <f aca="false">IFERROR(AA117/AA118,0)</f>
@@ -12753,7 +12815,7 @@
       </c>
       <c r="Z120" s="33" t="n">
         <f aca="false">Z41+Z48</f>
-        <v>0</v>
+        <v>167000</v>
       </c>
       <c r="AA120" s="33" t="n">
         <f aca="false">AA41+AA48</f>
@@ -12882,7 +12944,7 @@
       </c>
       <c r="Z121" s="33" t="n">
         <f aca="false">Z44+Z51</f>
-        <v>0</v>
+        <v>334</v>
       </c>
       <c r="AA121" s="33" t="n">
         <f aca="false">AA44+AA51</f>
@@ -13011,7 +13073,7 @@
       </c>
       <c r="Z122" s="33" t="n">
         <f aca="false">IFERROR(Z120/Z121,0)</f>
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="AA122" s="33" t="n">
         <f aca="false">IFERROR(AA120/AA121,0)</f>
@@ -13516,7 +13578,9 @@
       <c r="Y129" s="26" t="n">
         <v>984</v>
       </c>
-      <c r="Z129" s="26"/>
+      <c r="Z129" s="26" t="n">
+        <v>1461</v>
+      </c>
       <c r="AA129" s="26"/>
       <c r="AB129" s="26"/>
       <c r="AC129" s="26"/>
@@ -13558,7 +13622,9 @@
       <c r="Y130" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="Z130" s="26"/>
+      <c r="Z130" s="26" t="n">
+        <v>3</v>
+      </c>
       <c r="AA130" s="26"/>
       <c r="AB130" s="26"/>
       <c r="AC130" s="26"/>
@@ -13584,7 +13650,9 @@
       <c r="Y131" s="26" t="n">
         <v>607.33</v>
       </c>
-      <c r="Z131" s="26"/>
+      <c r="Z131" s="26" t="n">
+        <v>610.33</v>
+      </c>
       <c r="AA131" s="26"/>
       <c r="AB131" s="26"/>
       <c r="AC131" s="26"/>
@@ -13656,7 +13724,9 @@
       <c r="Y132" s="26" t="n">
         <v>13318</v>
       </c>
-      <c r="Z132" s="26"/>
+      <c r="Z132" s="26" t="n">
+        <v>13970</v>
+      </c>
       <c r="AA132" s="26"/>
       <c r="AB132" s="26"/>
       <c r="AC132" s="26"/>
@@ -13728,7 +13798,9 @@
       <c r="Y133" s="37" t="n">
         <v>0.022</v>
       </c>
-      <c r="Z133" s="37"/>
+      <c r="Z133" s="37" t="n">
+        <v>0.022</v>
+      </c>
       <c r="AA133" s="37"/>
       <c r="AB133" s="37"/>
       <c r="AC133" s="37"/>
@@ -14022,7 +14094,9 @@
       <c r="X5" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="Y5" s="42"/>
+      <c r="Y5" s="42" t="s">
+        <v>118</v>
+      </c>
       <c r="Z5" s="42"/>
       <c r="AA5" s="42"/>
       <c r="AB5" s="42"/>
@@ -14034,7 +14108,7 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="41" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C6" s="42"/>
       <c r="D6" s="42"/>
@@ -14055,14 +14129,16 @@
       <c r="S6" s="42"/>
       <c r="T6" s="42"/>
       <c r="U6" s="42" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="V6" s="42"/>
       <c r="W6" s="42"/>
       <c r="X6" s="42" t="s">
-        <v>120</v>
-      </c>
-      <c r="Y6" s="42"/>
+        <v>121</v>
+      </c>
+      <c r="Y6" s="42" t="s">
+        <v>122</v>
+      </c>
       <c r="Z6" s="42"/>
       <c r="AA6" s="42"/>
       <c r="AB6" s="42"/>
@@ -14074,7 +14150,7 @@
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="43" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C7" s="43"/>
       <c r="D7" s="43"/>
@@ -14098,7 +14174,7 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="41" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="44"/>
@@ -14119,14 +14195,16 @@
       <c r="S8" s="44"/>
       <c r="T8" s="44"/>
       <c r="U8" s="44" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="V8" s="44"/>
       <c r="W8" s="44"/>
       <c r="X8" s="44" t="s">
-        <v>124</v>
-      </c>
-      <c r="Y8" s="44"/>
+        <v>126</v>
+      </c>
+      <c r="Y8" s="44" t="s">
+        <v>127</v>
+      </c>
       <c r="Z8" s="44"/>
       <c r="AA8" s="44"/>
       <c r="AB8" s="44"/>
@@ -14138,7 +14216,7 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="41" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C9" s="44"/>
       <c r="D9" s="44"/>
@@ -14159,14 +14237,16 @@
       <c r="S9" s="44"/>
       <c r="T9" s="44"/>
       <c r="U9" s="44" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="V9" s="44"/>
       <c r="W9" s="44"/>
       <c r="X9" s="44" t="s">
-        <v>127</v>
-      </c>
-      <c r="Y9" s="44"/>
+        <v>130</v>
+      </c>
+      <c r="Y9" s="44" t="s">
+        <v>131</v>
+      </c>
       <c r="Z9" s="44"/>
       <c r="AA9" s="44"/>
       <c r="AB9" s="44"/>
@@ -14178,7 +14258,7 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="41" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C10" s="44"/>
       <c r="D10" s="44"/>
@@ -14199,14 +14279,16 @@
       <c r="S10" s="44"/>
       <c r="T10" s="44"/>
       <c r="U10" s="44" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="V10" s="44"/>
       <c r="W10" s="44"/>
       <c r="X10" s="44" t="s">
-        <v>130</v>
-      </c>
-      <c r="Y10" s="44"/>
+        <v>134</v>
+      </c>
+      <c r="Y10" s="44" t="s">
+        <v>135</v>
+      </c>
       <c r="Z10" s="44"/>
       <c r="AA10" s="44"/>
       <c r="AB10" s="44"/>
@@ -14218,7 +14300,7 @@
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="45" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C11" s="45"/>
       <c r="D11" s="45"/>
@@ -14242,7 +14324,7 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="41" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C12" s="46"/>
       <c r="D12" s="46"/>
@@ -14263,14 +14345,16 @@
       <c r="S12" s="46"/>
       <c r="T12" s="46"/>
       <c r="U12" s="46" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="V12" s="46"/>
       <c r="W12" s="46"/>
       <c r="X12" s="46" t="s">
-        <v>134</v>
-      </c>
-      <c r="Y12" s="46"/>
+        <v>139</v>
+      </c>
+      <c r="Y12" s="46" t="s">
+        <v>140</v>
+      </c>
       <c r="Z12" s="46"/>
       <c r="AA12" s="46"/>
       <c r="AB12" s="46"/>
@@ -14282,7 +14366,7 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="41" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="C13" s="46"/>
       <c r="D13" s="46"/>
@@ -14303,12 +14387,12 @@
       <c r="S13" s="46"/>
       <c r="T13" s="46"/>
       <c r="U13" s="46" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="V13" s="46"/>
       <c r="W13" s="46"/>
       <c r="X13" s="46" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="Y13" s="46"/>
       <c r="Z13" s="46"/>
@@ -14322,7 +14406,7 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="41" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="C14" s="46"/>
       <c r="D14" s="46"/>
@@ -14343,7 +14427,7 @@
       <c r="S14" s="46"/>
       <c r="T14" s="46"/>
       <c r="U14" s="46" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="V14" s="46"/>
       <c r="W14" s="46"/>
@@ -14360,7 +14444,7 @@
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="47" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="C15" s="47"/>
       <c r="D15" s="47"/>
@@ -14384,7 +14468,7 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="41" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C16" s="48"/>
       <c r="D16" s="48"/>
@@ -14405,14 +14489,16 @@
       <c r="S16" s="48"/>
       <c r="T16" s="48"/>
       <c r="U16" s="48" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="V16" s="48"/>
       <c r="W16" s="48"/>
       <c r="X16" s="48" t="s">
-        <v>143</v>
-      </c>
-      <c r="Y16" s="48"/>
+        <v>149</v>
+      </c>
+      <c r="Y16" s="48" t="s">
+        <v>150</v>
+      </c>
       <c r="Z16" s="48"/>
       <c r="AA16" s="48"/>
       <c r="AB16" s="48"/>
@@ -14424,7 +14510,7 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="41" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C17" s="48"/>
       <c r="D17" s="48"/>
@@ -14445,14 +14531,16 @@
       <c r="S17" s="48"/>
       <c r="T17" s="48"/>
       <c r="U17" s="48" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="V17" s="48"/>
       <c r="W17" s="48"/>
       <c r="X17" s="48" t="s">
-        <v>146</v>
-      </c>
-      <c r="Y17" s="48"/>
+        <v>153</v>
+      </c>
+      <c r="Y17" s="48" t="s">
+        <v>154</v>
+      </c>
       <c r="Z17" s="48"/>
       <c r="AA17" s="48"/>
       <c r="AB17" s="48"/>
@@ -14464,7 +14552,7 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="49" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="C18" s="49"/>
       <c r="D18" s="49"/>
@@ -14488,7 +14576,7 @@
     </row>
     <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="41" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
@@ -14509,12 +14597,12 @@
       <c r="S19" s="50"/>
       <c r="T19" s="50"/>
       <c r="U19" s="50" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="V19" s="50"/>
       <c r="W19" s="50"/>
       <c r="X19" s="50" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="Y19" s="50"/>
       <c r="Z19" s="50"/>
@@ -14528,7 +14616,7 @@
     </row>
     <row r="20" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="41" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="C20" s="50"/>
       <c r="D20" s="50"/>
@@ -14549,12 +14637,12 @@
       <c r="S20" s="50"/>
       <c r="T20" s="50"/>
       <c r="U20" s="50" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="V20" s="50"/>
       <c r="W20" s="50"/>
       <c r="X20" s="50" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="Y20" s="50"/>
       <c r="Z20" s="50"/>
@@ -14568,7 +14656,7 @@
     </row>
     <row r="21" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="41" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C21" s="50"/>
       <c r="D21" s="50"/>
@@ -14589,12 +14677,12 @@
       <c r="S21" s="50"/>
       <c r="T21" s="50"/>
       <c r="U21" s="50" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="V21" s="50"/>
       <c r="W21" s="50"/>
       <c r="X21" s="50" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="Y21" s="50"/>
       <c r="Z21" s="50"/>
@@ -14639,7 +14727,7 @@
     <row r="1" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="51" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
@@ -14672,7 +14760,7 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="52" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="C3" s="52"/>
       <c r="D3" s="52"/>
@@ -14693,7 +14781,7 @@
       <c r="S3" s="52"/>
       <c r="V3" s="53" t="str">
         <f aca="true">TEXT(Input!V$3,"mmmm yyyy")&amp;" · Prepared "&amp;TEXT(TODAY(),"mmm d, yyyy")</f>
-        <v>March 2026 · Prepared Aug 2, 2026</v>
+        <v>March 2026 · Prepared Aug 5, 2026</v>
       </c>
       <c r="W3" s="53"/>
       <c r="X3" s="53"/>
@@ -14738,42 +14826,42 @@
     <row r="5" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="55" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C6" s="55"/>
       <c r="D6" s="55"/>
       <c r="E6" s="55"/>
       <c r="F6" s="55"/>
       <c r="G6" s="55" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="H6" s="55"/>
       <c r="I6" s="55"/>
       <c r="J6" s="55"/>
       <c r="K6" s="55"/>
       <c r="L6" s="55" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="M6" s="55"/>
       <c r="N6" s="55"/>
       <c r="O6" s="55"/>
       <c r="P6" s="55"/>
       <c r="Q6" s="55" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="R6" s="55"/>
       <c r="S6" s="55"/>
       <c r="T6" s="55"/>
       <c r="U6" s="55"/>
       <c r="V6" s="55" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="W6" s="55"/>
       <c r="X6" s="55"/>
       <c r="Y6" s="55"/>
       <c r="Z6" s="55"/>
       <c r="AA6" s="55" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="AB6" s="55"/>
       <c r="AC6" s="55"/>
@@ -14930,42 +15018,42 @@
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="66" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C10" s="66"/>
       <c r="D10" s="66"/>
       <c r="E10" s="66"/>
       <c r="F10" s="66"/>
       <c r="G10" s="66" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="H10" s="66"/>
       <c r="I10" s="66"/>
       <c r="J10" s="66"/>
       <c r="K10" s="66"/>
       <c r="L10" s="66" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="M10" s="66"/>
       <c r="N10" s="66"/>
       <c r="O10" s="66"/>
       <c r="P10" s="66"/>
       <c r="Q10" s="66" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="R10" s="66"/>
       <c r="S10" s="66"/>
       <c r="T10" s="66"/>
       <c r="U10" s="66"/>
       <c r="V10" s="66" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="W10" s="66"/>
       <c r="X10" s="66"/>
       <c r="Y10" s="66"/>
       <c r="Z10" s="66"/>
       <c r="AA10" s="66" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="AB10" s="66"/>
       <c r="AC10" s="66"/>
@@ -14976,7 +15064,7 @@
     <row r="12" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="67" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="C13" s="67"/>
       <c r="D13" s="67"/>
@@ -15029,7 +15117,7 @@
     <row r="33" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="67" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C34" s="67"/>
       <c r="D34" s="67"/>
@@ -15062,7 +15150,7 @@
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="68" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="C35" s="68"/>
       <c r="D35" s="68"/>
@@ -15074,7 +15162,7 @@
       <c r="J35" s="68"/>
       <c r="K35" s="68"/>
       <c r="L35" s="69" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="M35" s="69"/>
       <c r="N35" s="69"/>
@@ -15086,7 +15174,7 @@
       <c r="T35" s="69"/>
       <c r="U35" s="69"/>
       <c r="V35" s="70" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="W35" s="70"/>
       <c r="X35" s="70"/>
@@ -15515,7 +15603,7 @@
     <row r="51" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="38" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C52" s="38"/>
       <c r="D52" s="38"/>
@@ -15549,7 +15637,7 @@
     <row r="53" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="54" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="74" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C54" s="74"/>
       <c r="D54" s="74"/>
@@ -15557,37 +15645,37 @@
       <c r="F54" s="74"/>
       <c r="G54" s="74"/>
       <c r="H54" s="75" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="I54" s="75"/>
       <c r="J54" s="75"/>
       <c r="K54" s="75"/>
       <c r="L54" s="75" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="M54" s="75"/>
       <c r="N54" s="75" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="O54" s="75"/>
       <c r="P54" s="75"/>
       <c r="Q54" s="75" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="R54" s="75"/>
       <c r="S54" s="75"/>
       <c r="T54" s="75" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="U54" s="75"/>
       <c r="V54" s="75"/>
       <c r="W54" s="75" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="X54" s="75"/>
       <c r="Y54" s="75"/>
       <c r="Z54" s="75" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="AA54" s="75"/>
       <c r="AB54" s="75"/>
@@ -16147,7 +16235,7 @@
     </row>
     <row r="65" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="89" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C65" s="89"/>
       <c r="D65" s="89"/>
@@ -16190,7 +16278,7 @@
       <c r="X65" s="95"/>
       <c r="Y65" s="95"/>
       <c r="Z65" s="96" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="AA65" s="96"/>
       <c r="AB65" s="96"/>
@@ -16201,7 +16289,7 @@
     <row r="66" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="97" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="C67" s="97"/>
       <c r="D67" s="97"/>
@@ -16218,7 +16306,7 @@
       <c r="O67" s="97"/>
       <c r="P67" s="97"/>
       <c r="Q67" s="97" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="R67" s="97"/>
       <c r="S67" s="97"/>
@@ -16400,7 +16488,7 @@
     <row r="87" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="8" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C88" s="8"/>
       <c r="D88" s="8"/>
@@ -16433,7 +16521,7 @@
     </row>
     <row r="89" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="55" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C89" s="55"/>
       <c r="D89" s="55"/>
@@ -16442,7 +16530,7 @@
       <c r="G89" s="55"/>
       <c r="H89" s="55"/>
       <c r="I89" s="55" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="J89" s="55"/>
       <c r="K89" s="55"/>
@@ -16451,7 +16539,7 @@
       <c r="N89" s="55"/>
       <c r="O89" s="55"/>
       <c r="P89" s="55" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="Q89" s="55"/>
       <c r="R89" s="55"/>
@@ -16461,7 +16549,7 @@
       <c r="V89" s="55"/>
       <c r="W89" s="55"/>
       <c r="X89" s="55" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="Y89" s="55"/>
       <c r="Z89" s="55"/>
@@ -16544,7 +16632,7 @@
     </row>
     <row r="92" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="101" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="C92" s="101"/>
       <c r="D92" s="101"/>
@@ -16553,7 +16641,7 @@
       <c r="G92" s="101"/>
       <c r="H92" s="101"/>
       <c r="I92" s="101" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="J92" s="101"/>
       <c r="K92" s="101"/>
@@ -16562,7 +16650,7 @@
       <c r="N92" s="101"/>
       <c r="O92" s="101"/>
       <c r="P92" s="101" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="Q92" s="101"/>
       <c r="R92" s="101"/>
@@ -16572,7 +16660,7 @@
       <c r="V92" s="101"/>
       <c r="W92" s="101"/>
       <c r="X92" s="101" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="Y92" s="101"/>
       <c r="Z92" s="101"/>
@@ -16583,7 +16671,7 @@
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B94" s="102" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="C94" s="102"/>
       <c r="D94" s="102"/>
@@ -16655,7 +16743,7 @@
     <row r="101" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="102" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B102" s="38" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C102" s="38"/>
       <c r="D102" s="38"/>
@@ -16688,7 +16776,7 @@
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B104" s="67" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C104" s="67"/>
       <c r="D104" s="67"/>
@@ -16705,7 +16793,7 @@
       <c r="O104" s="67"/>
       <c r="P104" s="67"/>
       <c r="Q104" s="67" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="R104" s="67"/>
       <c r="S104" s="67"/>
@@ -16723,42 +16811,42 @@
     </row>
     <row r="106" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B106" s="104" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C106" s="104"/>
       <c r="D106" s="104"/>
       <c r="E106" s="104"/>
       <c r="F106" s="104" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="G106" s="104"/>
       <c r="H106" s="104"/>
       <c r="I106" s="104"/>
       <c r="J106" s="104" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="K106" s="104"/>
       <c r="L106" s="104"/>
       <c r="M106" s="104"/>
       <c r="N106" s="104" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="O106" s="104"/>
       <c r="P106" s="104"/>
       <c r="Q106" s="104" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="R106" s="104"/>
       <c r="S106" s="104"/>
       <c r="T106" s="104"/>
       <c r="U106" s="104" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="V106" s="104"/>
       <c r="W106" s="104"/>
       <c r="X106" s="104"/>
       <c r="Y106" s="104" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="Z106" s="104"/>
       <c r="AA106" s="104"/>
@@ -16851,7 +16939,7 @@
     </row>
     <row r="110" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B110" s="109" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="C110" s="109"/>
       <c r="D110" s="109"/>
@@ -16868,7 +16956,7 @@
       <c r="O110" s="109"/>
       <c r="P110" s="109"/>
       <c r="Q110" s="109" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="R110" s="109"/>
       <c r="S110" s="109"/>
@@ -17163,7 +17251,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B137" s="113" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C137" s="113"/>
       <c r="D137" s="113"/>
@@ -17180,7 +17268,7 @@
       <c r="O137" s="113"/>
       <c r="P137" s="113"/>
       <c r="Q137" s="113" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="R137" s="113"/>
       <c r="S137" s="113"/>
@@ -17330,7 +17418,7 @@
     <row r="143" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="144" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B144" s="89" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="C144" s="89"/>
       <c r="D144" s="89"/>
@@ -17363,13 +17451,13 @@
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B145" s="114" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="C145" s="114"/>
       <c r="D145" s="114"/>
       <c r="E145" s="114"/>
       <c r="F145" s="115" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="G145" s="115"/>
       <c r="H145" s="115"/>
@@ -17382,13 +17470,13 @@
       <c r="O145" s="115"/>
       <c r="P145" s="115"/>
       <c r="Q145" s="114" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="R145" s="114"/>
       <c r="S145" s="114"/>
       <c r="T145" s="114"/>
       <c r="U145" s="115" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="V145" s="115"/>
       <c r="W145" s="115"/>
@@ -17402,13 +17490,13 @@
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B146" s="114" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="C146" s="114"/>
       <c r="D146" s="114"/>
       <c r="E146" s="114"/>
       <c r="F146" s="115" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="G146" s="115"/>
       <c r="H146" s="115"/>
@@ -17421,13 +17509,13 @@
       <c r="O146" s="115"/>
       <c r="P146" s="115"/>
       <c r="Q146" s="114" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="R146" s="114"/>
       <c r="S146" s="114"/>
       <c r="T146" s="114"/>
       <c r="U146" s="115" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="V146" s="115"/>
       <c r="W146" s="115"/>
@@ -17441,13 +17529,13 @@
     </row>
     <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B147" s="114" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="C147" s="114"/>
       <c r="D147" s="114"/>
       <c r="E147" s="114"/>
       <c r="F147" s="115" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="G147" s="115"/>
       <c r="H147" s="115"/>
@@ -17460,13 +17548,13 @@
       <c r="O147" s="115"/>
       <c r="P147" s="115"/>
       <c r="Q147" s="114" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="R147" s="114"/>
       <c r="S147" s="114"/>
       <c r="T147" s="114"/>
       <c r="U147" s="115" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="V147" s="115"/>
       <c r="W147" s="115"/>
@@ -17480,13 +17568,13 @@
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B148" s="114" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="C148" s="114"/>
       <c r="D148" s="114"/>
       <c r="E148" s="114"/>
       <c r="F148" s="115" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="G148" s="115"/>
       <c r="H148" s="115"/>
@@ -17499,13 +17587,13 @@
       <c r="O148" s="115"/>
       <c r="P148" s="115"/>
       <c r="Q148" s="114" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="R148" s="114"/>
       <c r="S148" s="114"/>
       <c r="T148" s="114"/>
       <c r="U148" s="115" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="V148" s="115"/>
       <c r="W148" s="115"/>
@@ -17519,7 +17607,7 @@
     </row>
     <row r="151" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B151" s="116" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="C151" s="116"/>
       <c r="D151" s="116"/>

</xml_diff>

<commit_message>
Juli 2026 final: kunder/maalepunkter, Tot CAC N/A, regningstjek-note
</commit_message>
<xml_diff>
--- a/AE-marketingrapport-master.xlsx
+++ b/AE-marketingrapport-master.xlsx
@@ -400,7 +400,7 @@
     <t xml:space="preserve">Sign-ups landede på 984, et forventet sæsonfald fra maj (1.035), men konverteringen steg igen — blended CVR ramte 6,4% mod 5,8% i maj. Google leverede 74 kunder til en CAC på 133 kr. (kanalens næstbedste måned), og Brand search fastholdt det høje niveau med 446 kunder. Churn faldt tilbage fra 2,6% til 2,2%, og vi rundede 13.318 aktive kunder (+582).</t>
   </si>
   <si>
-    <t xml:space="preserve">Juli blev den største måned i Altid Energis historie med 1.461 signups, klart over den tidligere rekord på 1.300 fra februar. Blended konvertering ramte 10,0 pct. (ny rekord), og blended CAC faldt til 131 kr. fra 157 kr. Brand search leverede 733 kunder (rekord), Google sin bedste konverteringsmåned (CVR 11,1 pct., CAC 105 kr.), og affiliates voksede til 334 kunder. Aktive kunder rundede 13.970 (+652), og churn holdt sig stabil på 2,2 pct.</t>
+    <t xml:space="preserve">Juli blev den største måned i Altid Energis historie med 1.461 signups, klart over den tidligere rekord på 1.300 fra februar. Blended konvertering ramte 10,0 pct. (ny rekord), og blended CAC faldt til 131 kr. fra 157 kr. Brand search leverede 733 kunder (rekord), Google sin bedste konverteringsmåned (CVR 11,1 pct., CAC 105 kr.), og affiliates voksede til 334 kunder. Aktive kunder rundede 13.970 (15.267 målepunkter) med en nettotilvækst på 652, og churn holdt sig stabil på 2,2 pct.</t>
   </si>
   <si>
     <t xml:space="preserve">WINS — HVAD VIRKEDE</t>
@@ -2129,8 +2129,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86917899"/>
-        <c:axId val="31025123"/>
+        <c:axId val="2157835"/>
+        <c:axId val="41765347"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2315,11 +2315,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="4644969"/>
-        <c:axId val="16117395"/>
+        <c:axId val="57907455"/>
+        <c:axId val="93378071"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="86917899"/>
+        <c:axId val="2157835"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2350,7 +2350,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31025123"/>
+        <c:crossAx val="41765347"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -2358,7 +2358,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="31025123"/>
+        <c:axId val="41765347"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2423,12 +2423,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86917899"/>
+        <c:crossAx val="2157835"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:dateAx>
-        <c:axId val="4644969"/>
+        <c:axId val="57907455"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2459,7 +2459,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16117395"/>
+        <c:crossAx val="93378071"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -2467,7 +2467,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="16117395"/>
+        <c:axId val="93378071"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2532,7 +2532,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4644969"/>
+        <c:crossAx val="57907455"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2747,11 +2747,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71657506"/>
-        <c:axId val="24797220"/>
+        <c:axId val="55411938"/>
+        <c:axId val="98172424"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71657506"/>
+        <c:axId val="55411938"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2782,7 +2782,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24797220"/>
+        <c:crossAx val="98172424"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2790,7 +2790,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24797220"/>
+        <c:axId val="98172424"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2821,7 +2821,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71657506"/>
+        <c:crossAx val="55411938"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3012,11 +3012,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="84131102"/>
-        <c:axId val="57461450"/>
+        <c:axId val="78381551"/>
+        <c:axId val="33279198"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="84131102"/>
+        <c:axId val="78381551"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3047,7 +3047,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57461450"/>
+        <c:crossAx val="33279198"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3055,7 +3055,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="57461450"/>
+        <c:axId val="33279198"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3095,7 +3095,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84131102"/>
+        <c:crossAx val="78381551"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3347,11 +3347,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78426142"/>
-        <c:axId val="93029554"/>
+        <c:axId val="12541057"/>
+        <c:axId val="33098113"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="78426142"/>
+        <c:axId val="12541057"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3382,7 +3382,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93029554"/>
+        <c:crossAx val="33098113"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -3390,7 +3390,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="93029554"/>
+        <c:axId val="33098113"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3421,7 +3421,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78426142"/>
+        <c:crossAx val="12541057"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3673,11 +3673,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="46415980"/>
-        <c:axId val="59975435"/>
+        <c:axId val="82519521"/>
+        <c:axId val="60501339"/>
       </c:lineChart>
       <c:dateAx>
-        <c:axId val="46415980"/>
+        <c:axId val="82519521"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3708,7 +3708,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59975435"/>
+        <c:crossAx val="60501339"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
@@ -3716,7 +3716,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:dateAx>
       <c:valAx>
-        <c:axId val="59975435"/>
+        <c:axId val="60501339"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3747,7 +3747,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46415980"/>
+        <c:crossAx val="82519521"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3786,9 +3786,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
-      <xdr:colOff>221760</xdr:colOff>
+      <xdr:colOff>221040</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>101880</xdr:rowOff>
+      <xdr:rowOff>101160</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3797,7 +3797,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="293400" y="2114640"/>
-        <a:ext cx="9633600" cy="2330640"/>
+        <a:ext cx="9632880" cy="2329920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3816,9 +3816,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>231840</xdr:colOff>
+      <xdr:colOff>231120</xdr:colOff>
       <xdr:row>81</xdr:row>
-      <xdr:rowOff>63720</xdr:rowOff>
+      <xdr:rowOff>63000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3827,7 +3827,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="293400" y="11458440"/>
-        <a:ext cx="4632480" cy="2330640"/>
+        <a:ext cx="4631760" cy="2329920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3846,9 +3846,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>232200</xdr:colOff>
+      <xdr:colOff>231480</xdr:colOff>
       <xdr:row>81</xdr:row>
-      <xdr:rowOff>63720</xdr:rowOff>
+      <xdr:rowOff>63000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3857,7 +3857,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4694040" y="11458440"/>
-        <a:ext cx="4632480" cy="2330640"/>
+        <a:ext cx="4631760" cy="2329920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3876,9 +3876,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>231840</xdr:colOff>
+      <xdr:colOff>231120</xdr:colOff>
       <xdr:row>123</xdr:row>
-      <xdr:rowOff>151200</xdr:rowOff>
+      <xdr:rowOff>150480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3887,7 +3887,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="293400" y="18773640"/>
-        <a:ext cx="4632480" cy="1608840"/>
+        <a:ext cx="4631760" cy="1608120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3906,9 +3906,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>232200</xdr:colOff>
+      <xdr:colOff>231480</xdr:colOff>
       <xdr:row>123</xdr:row>
-      <xdr:rowOff>151200</xdr:rowOff>
+      <xdr:rowOff>150480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3917,7 +3917,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="4694040" y="18773640"/>
-        <a:ext cx="4632480" cy="1608840"/>
+        <a:ext cx="4631760" cy="1608120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">

</xml_diff>